<commit_message>
Restructured repository organistation - FLoRA gen is working, FReD not yet
</commit_message>
<xml_diff>
--- a/archive/quote mismatch.xlsx
+++ b/archive/quote mismatch.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -372,243 +372,63 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>study_o</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>ref_r</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>doi_r</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>url_r</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>link_r</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>study_r</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>abstract_r</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>entries_per_rep</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>success_rating</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>success_quote</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>quote_detect</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>quote_dist</t>
         </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>additional_studies36</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Sfärlea, A., Greimel, E., Platt, B., Dieler, A. C., &amp; Schulte‐Körne, G. (2018). Recognition of emotional facial expressions in adolescents with anorexia nervosa and adolescents with major depression. Psychiatry Research, 262, 586–594.</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>10.1016/j.psychres.2017.09.048</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Sfärlea, A., Buhl, C., Lukas, L., &amp; Schulte‐Körne, G. (2024). Superior facial emotion recognition in adolescents with anorexia nervosa–A replication study. European Eating Disorders Review.</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>10.1002/erv.3103</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1bJ0BC-Xy_bNt41DXHAjv1ms0mnz9Vq86/view?usp=drivesdk</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>AbstractObjectiveAnorexia nervosa (AN) has been associated with alterations in the processing of socio‐emotional information, including impairments in the recognition of emotions in other people's faces. However, adolescents with AN might not show the impairments found in adult patients. The present study investigated facial emotion recognition in adolescents with AN, aiming to replicate our previous results of superior emotion recognition abilities in adolescents with AN compared to adolescents without mental disorders.Method
-                      Adolescent girls (12–18 years) with AN (
-                      n
-                       = 33) were compared to girls without mental disorders (
-                      n
-                       = 41). Participants completed one task requiring identification of emotions (happy, sad, afraid, angry, neutral) in faces and one control task.
-                    ResultsAs expected, adolescents with AN showed superior emotion recognition, with higher accuracy rates specifically for afraid faces.ConclusionThis is the first study replicating previous results on basic emotion recognition in adolescents with AN using (almost) the same methodology. The results suggest that, in contrast to adults, adolescents with AN do not show impairments in facial emotion recognition. The impairments may arise in the longer course of the illness, however, longitudinal studies are necessary to confirm this assumption.</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>successful</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>As expected, adolescents with AN showed superior emotion recognition, with higher accuracy rates specifically for afraid faces. This is the first study replicating previous results on basic emotion recognition in adolescents with AN using (almost) the same methodology.</t>
-        </is>
-      </c>
-      <c r="L2" t="b">
-        <v>0</v>
-      </c>
-      <c r="M2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>additional_studies37</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Rothman, J. (2011). L3 syntactic transfer selectivity and typological determinacy: The typological primacy model. Second Language Research, 27, 107–127.</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>10.1177/0267658310386439</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Parrish, K. (2024). Statistical Insignificance is not wholesale transfer in L3 Acquisition: an approximate replication of Rothman (2011). Studies in Second Language Acquisition, 1-18.</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>10.1017/S0272263124000342</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1fNwzy4f6SEAeVccICF8BD0SDAIH7uPVr/view?usp=drivesdk</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Abstract
-                    This study was an approximate replication of Rothman (2011),examining the determiner phrase syntax of a large sample (
-                    n
-                    = 211) of L3 learners of Portuguese who spoke English and Spanish. Rothman (2011) investigated whether L3 Italian or Brazilian Portuguese speakers are differently impacted by another known Romance Language, if it was their L1 or L2. The original study concluded that groups did not perform differently on experimental tasks on the basis of a null effect, and that the typological similarity of Spanish, Portuguese, or Italian predicts transfer in the initial stages of L3 acquisition. The present replication recreated all materials, which were unavailable, and examined the same population and questions. However, rather than examining L3 Italian and L3 Brazilian Portuguese, the present work maintained a constant L3 Portuguese. Learners were divided into two groups in a mirror-image design (
-                    n
-                    = 96 L1 English-L2 Spanish,
-                    n
-                    = 115 L1 Spanish-L2 English), and data were collected online. Like the original study, there was no main effect of group in any of the two-way analyses of variance. However, results show that it should not be assumed that experimental groups behave equivalently based on a null effect: Of the four total post hoc tests of equivalence, only two were significant when the equivalence bounds were set at a small effect size (d =
-                    $ \pm $
-                    .4). Ultimately, it is argued that determining the smallest effect size of interest and subsequent equivalence testing are necessary to answer key questions in the field of L3 acquisition.
-                  </t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>statistically successful but highlighting fundamental flaws</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Like the original study, there was no main effect of group in any of the two-way analyses of variance. However, results show that it should not be assumed that experimental groups behave equivalently based on a null effect: Of the four total post hoc tests of equivalence, only two were significant when the equivalence bounds were set at a small effect size (d = ± .4).</t>
-        </is>
-      </c>
-      <c r="L3" t="b">
-        <v>0</v>
-      </c>
-      <c r="M3">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>additional_studies240</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Iyengar, S., Kinder, D. R., Peters, M. D., &amp; Krosnick, J. A. (1984). The evening news and presidential evaluations. Journal of personality and social psychology, 46(4), 778. https://psycnet.apa.org/doi/10.1037/0022-3514.46.4.778</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>10.1037/0022-3514.46.4.778</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Kobayashi, T., Miura, A., &amp; Inamasu, K. (2017). Media Priming Effect: A Preregistered Replication Experiment. Journal of Experimental Political Science, 4(1), 81–94.</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>10.1017/XPS.2017.8</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1aV3ccn2w0Qw9IRbsqbByGUHxTunteFgK/view?usp=drivesdk</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>AbstractIyengar et al. (1984, The Evening News and Presidential Evaluations. Journal of Personality and Social Psychology 46(4): 778–87) discovered the media priming effect, positing that by drawing attention to certain issues while ignoring others, television news programs help define the standards by which presidents are evaluated. We conducted a direct replication of Experiment 1 by Iyengar et al. (1984, The Evening News and Presidential Evaluations. Journal of Personality and Social Psychology 46(4): 778–87) with some changes. Specifically, we (a) collected data from Japanese undergraduates; (b) reduced the number of conditions to two; (c) used news coverage of the issue of relocating US bases in Okinawa as the treatment; (d) measured issue-specific evaluations of the Japanese Prime Minister in the pre-treatment questionnaire; and (e) performed statistical analyses that are more appropriate for testing heterogeneity in the treatment effect. We did not find statistically significant evidence of media priming. Overall, the results suggest that the effects of media priming may be quite sensitive either to the media environment or to differences in populations in which the effect has been examined.</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>failed</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Iyengar et al. (1984) discovered the media priming effect [...] We did not find statistically significant evidence of media priming.</t>
-        </is>
-      </c>
-      <c r="L4" t="b">
-        <v>0</v>
-      </c>
-      <c r="M4">
-        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>